<commit_message>
Added NorthwindTablesAndColumns.xlsx // Ex_2b
</commit_message>
<xml_diff>
--- a/week-09/NorthwindTablesAndColumns.xlsx
+++ b/week-09/NorthwindTablesAndColumns.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://reliablecollaboration-my.sharepoint.com/personal/bess_rcc_team/Documents/Courseware/DataAnalyst_Spring2026_SharedWithPS/Week 9 - Getting Started with Power BI/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luise\Documents\DataAnalytics\week-09\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{FA878EF4-4B80-439A-88BC-05CECC90D1C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47F2F594-F8DE-4E97-9375-0231B9F751D4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D87DD04-47C3-4DD6-8907-99C977B5468B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27465" yWindow="360" windowWidth="21120" windowHeight="20040" xr2:uid="{901F5D27-877F-4C94-89AE-9A9B6ECE5CB6}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{901F5D27-877F-4C94-89AE-9A9B6ECE5CB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Northwind Columns" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="144">
   <si>
     <t>table_name</t>
   </si>
@@ -308,6 +308,165 @@
   </si>
   <si>
     <t>New Column Name?</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Company Contact</t>
+  </si>
+  <si>
+    <t>Customer City</t>
+  </si>
+  <si>
+    <t>Customer Region</t>
+  </si>
+  <si>
+    <t>Customer Country</t>
+  </si>
+  <si>
+    <t>Employee Title</t>
+  </si>
+  <si>
+    <t>Employee City</t>
+  </si>
+  <si>
+    <t>Employee Region</t>
+  </si>
+  <si>
+    <t>Employee Country</t>
+  </si>
+  <si>
+    <t>Customer Postal</t>
+  </si>
+  <si>
+    <t>Employee Last Name</t>
+  </si>
+  <si>
+    <t>Employee First Name</t>
+  </si>
+  <si>
+    <t>Employee Title Of Courtesy</t>
+  </si>
+  <si>
+    <t>Employee Birth Date</t>
+  </si>
+  <si>
+    <t>Employee Hire Date</t>
+  </si>
+  <si>
+    <t>Employee Postal Code</t>
+  </si>
+  <si>
+    <t>Employee Reports To</t>
+  </si>
+  <si>
+    <t>Supplier Contact Name</t>
+  </si>
+  <si>
+    <t>Supplier Contact Title</t>
+  </si>
+  <si>
+    <t>Supplier City</t>
+  </si>
+  <si>
+    <t>Supplier Region</t>
+  </si>
+  <si>
+    <t>Supplier Postal Code</t>
+  </si>
+  <si>
+    <t>Supplier Country</t>
+  </si>
+  <si>
+    <t>Order Unit Price</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Product Unit Price</t>
+  </si>
+  <si>
+    <t>Products On Order</t>
+  </si>
+  <si>
+    <t>Products In Stock</t>
+  </si>
+  <si>
+    <t>Order Quantity</t>
+  </si>
+  <si>
+    <t>Order Discount Percentage</t>
+  </si>
+  <si>
+    <t>Order Date</t>
+  </si>
+  <si>
+    <t>Order Required Date</t>
+  </si>
+  <si>
+    <t>Order Shipped Date</t>
+  </si>
+  <si>
+    <t>Order Ship Via</t>
+  </si>
+  <si>
+    <t>Order Ship Name</t>
+  </si>
+  <si>
+    <t>Order Ship City</t>
+  </si>
+  <si>
+    <t>Order Ship Region</t>
+  </si>
+  <si>
+    <t>Order Ship Country</t>
+  </si>
+  <si>
+    <t>Order Ship Postal</t>
+  </si>
+  <si>
+    <t>Products Qty per Unit</t>
+  </si>
+  <si>
+    <t>Product Reorder Level</t>
+  </si>
+  <si>
+    <t>Shipper</t>
+  </si>
+  <si>
+    <t>Supplier</t>
+  </si>
+  <si>
+    <t>COUNT</t>
+  </si>
+  <si>
+    <t>Company Contact Title</t>
+  </si>
+  <si>
+    <t>SUM</t>
+  </si>
+  <si>
+    <t>MULTI AGGREGATIONS</t>
+  </si>
+  <si>
+    <t>AVG</t>
+  </si>
+  <si>
+    <t>Can first and last name be combined?</t>
+  </si>
+  <si>
+    <t>Is title of courtesy necessary to keep?</t>
   </si>
 </sst>
 </file>
@@ -371,11 +530,13 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="3"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent1" xfId="1" builtinId="30"/>
@@ -694,23 +855,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6B56A5E-AA28-4DB9-BAE3-51DE131C631E}">
   <dimension ref="A1:N85"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" customWidth="1"/>
-    <col min="9" max="9" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.84375" customWidth="1"/>
+    <col min="2" max="2" width="10.3046875" customWidth="1"/>
+    <col min="3" max="3" width="17.15234375" customWidth="1"/>
+    <col min="4" max="4" width="9.84375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.3828125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.3046875" customWidth="1"/>
+    <col min="7" max="7" width="17.84375" customWidth="1"/>
+    <col min="9" max="9" width="19.3828125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.84375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="26" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.5703125" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" customWidth="1"/>
+    <col min="12" max="12" width="15.53515625" customWidth="1"/>
+    <col min="13" max="13" width="11.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -754,7 +915,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -770,8 +931,26 @@
       <c r="E2" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F2" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -787,8 +966,32 @@
       <c r="E3" s="1">
         <v>30</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F3" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -804,8 +1007,26 @@
       <c r="E4" s="1">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F4" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -821,8 +1042,26 @@
       <c r="E5" s="1">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F5" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
@@ -838,8 +1077,26 @@
       <c r="E6" s="2">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F6" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
@@ -855,8 +1112,32 @@
       <c r="E7" s="2">
         <v>80</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F7" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
@@ -872,8 +1153,32 @@
       <c r="E8" s="2">
         <v>60</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F8" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -889,8 +1194,30 @@
       <c r="E9" s="2">
         <v>60</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F9" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M9" s="1"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
@@ -906,8 +1233,26 @@
       <c r="E10" s="2">
         <v>120</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F10" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>16</v>
       </c>
@@ -923,8 +1268,32 @@
       <c r="E11" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F11" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>16</v>
       </c>
@@ -940,8 +1309,32 @@
       <c r="E12" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F12" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>16</v>
       </c>
@@ -957,8 +1350,30 @@
       <c r="E13" s="2">
         <v>20</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F13" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M13" s="1"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
@@ -974,8 +1389,32 @@
       <c r="E14" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F14" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>16</v>
       </c>
@@ -991,8 +1430,26 @@
       <c r="E15" s="2">
         <v>48</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F15" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
@@ -1008,8 +1465,26 @@
       <c r="E16" s="2">
         <v>48</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L16" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
@@ -1025,8 +1500,26 @@
       <c r="E17" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
@@ -1042,8 +1535,35 @@
       <c r="E18" s="1">
         <v>40</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
@@ -1059,8 +1579,35 @@
       <c r="E19" s="1">
         <v>20</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L19" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
         <v>27</v>
       </c>
@@ -1076,8 +1623,29 @@
       <c r="E20" s="1">
         <v>60</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -1093,8 +1661,32 @@
       <c r="E21" s="1">
         <v>50</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
         <v>27</v>
       </c>
@@ -1110,8 +1702,29 @@
       <c r="E22" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A23" s="1" t="s">
         <v>27</v>
       </c>
@@ -1127,8 +1740,29 @@
       <c r="E23" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
         <v>27</v>
       </c>
@@ -1144,8 +1778,27 @@
       <c r="E24" s="1">
         <v>120</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I24" s="4"/>
+      <c r="J24" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
         <v>27</v>
       </c>
@@ -1161,8 +1814,32 @@
       <c r="E25" s="1">
         <v>30</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L25" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M25" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
         <v>27</v>
       </c>
@@ -1178,8 +1855,32 @@
       <c r="E26" s="1">
         <v>30</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M26" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
@@ -1195,8 +1896,29 @@
       <c r="E27" s="1">
         <v>20</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L27" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
         <v>27</v>
       </c>
@@ -1212,8 +1934,32 @@
       <c r="E28" s="1">
         <v>30</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F28" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M28" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -1229,8 +1975,27 @@
       <c r="E29" s="1">
         <v>48</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I29" s="4"/>
+      <c r="J29" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L29" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A30" s="1" t="s">
         <v>27</v>
       </c>
@@ -1246,8 +2011,27 @@
       <c r="E30" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I30" s="4"/>
+      <c r="J30" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A31" s="1" t="s">
         <v>27</v>
       </c>
@@ -1263,8 +2047,27 @@
       <c r="E31" s="1">
         <v>16</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F31" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I31" s="4"/>
+      <c r="J31" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L31" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A32" s="1" t="s">
         <v>27</v>
       </c>
@@ -1280,8 +2083,27 @@
       <c r="E32" s="1">
         <v>16</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F32" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I32" s="4"/>
+      <c r="J32" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A33" s="1" t="s">
         <v>27</v>
       </c>
@@ -1297,8 +2119,32 @@
       <c r="E33" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K33" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L33" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M33" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
         <v>27</v>
       </c>
@@ -1314,8 +2160,27 @@
       <c r="E34" s="1">
         <v>510</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F34" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I34" s="4"/>
+      <c r="J34" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K34" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L34" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A35" s="2" t="s">
         <v>42</v>
       </c>
@@ -1331,8 +2196,27 @@
       <c r="E35" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F35" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I35" s="4"/>
+      <c r="J35" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K35" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A36" s="2" t="s">
         <v>42</v>
       </c>
@@ -1348,8 +2232,27 @@
       <c r="E36" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F36" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I36" s="4"/>
+      <c r="J36" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L36" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A37" s="1" t="s">
         <v>44</v>
       </c>
@@ -1365,8 +2268,27 @@
       <c r="E37" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I37" s="4"/>
+      <c r="J37" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K37" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A38" s="1" t="s">
         <v>44</v>
       </c>
@@ -1382,8 +2304,27 @@
       <c r="E38" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F38" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I38" s="4"/>
+      <c r="J38" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K38" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L38" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A39" s="1" t="s">
         <v>44</v>
       </c>
@@ -1399,8 +2340,32 @@
       <c r="E39" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K39" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L39" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="M39" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A40" s="1" t="s">
         <v>44</v>
       </c>
@@ -1416,8 +2381,32 @@
       <c r="E40" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L40" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M40" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A41" s="1" t="s">
         <v>44</v>
       </c>
@@ -1433,8 +2422,32 @@
       <c r="E41" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F41" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K41" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L41" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="M41" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A42" s="2" t="s">
         <v>53</v>
       </c>
@@ -1450,8 +2463,26 @@
       <c r="E42" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F42" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K42" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L42" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A43" s="2" t="s">
         <v>53</v>
       </c>
@@ -1467,8 +2498,26 @@
       <c r="E43" s="2">
         <v>10</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F43" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G43" t="s">
+        <v>91</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J43" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K43" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L43" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A44" s="2" t="s">
         <v>53</v>
       </c>
@@ -1484,8 +2533,26 @@
       <c r="E44" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F44" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G44" t="s">
+        <v>91</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J44" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K44" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L44" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A45" s="2" t="s">
         <v>53</v>
       </c>
@@ -1501,8 +2568,32 @@
       <c r="E45" s="2">
         <v>8</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F45" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H45" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="J45" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K45" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L45" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M45" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A46" s="2" t="s">
         <v>53</v>
       </c>
@@ -1518,8 +2609,32 @@
       <c r="E46" s="2">
         <v>8</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F46" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M46" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A47" s="2" t="s">
         <v>53</v>
       </c>
@@ -1535,8 +2650,32 @@
       <c r="E47" s="2">
         <v>8</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F47" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="J47" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K47" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L47" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M47" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A48" s="2" t="s">
         <v>53</v>
       </c>
@@ -1552,8 +2691,32 @@
       <c r="E48" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F48" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I48" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="J48" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K48" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L48" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M48" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A49" s="2" t="s">
         <v>53</v>
       </c>
@@ -1569,8 +2732,27 @@
       <c r="E49" s="2">
         <v>8</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F49" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H49" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I49" s="5"/>
+      <c r="J49" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K49" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L49" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A50" s="2" t="s">
         <v>53</v>
       </c>
@@ -1586,8 +2768,32 @@
       <c r="E50" s="2">
         <v>80</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F50" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H50" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I50" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="J50" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K50" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L50" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M50" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A51" s="2" t="s">
         <v>53</v>
       </c>
@@ -1603,8 +2809,27 @@
       <c r="E51" s="2">
         <v>120</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F51" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H51" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I51" s="5"/>
+      <c r="J51" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K51" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L51" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A52" s="2" t="s">
         <v>53</v>
       </c>
@@ -1620,8 +2845,32 @@
       <c r="E52" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F52" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I52" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L52" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M52" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A53" s="2" t="s">
         <v>53</v>
       </c>
@@ -1637,8 +2886,32 @@
       <c r="E53" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F53" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H53" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I53" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="J53" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K53" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L53" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M53" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A54" s="2" t="s">
         <v>53</v>
       </c>
@@ -1654,8 +2927,29 @@
       <c r="E54" s="2">
         <v>20</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F54" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I54" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="J54" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L54" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
@@ -1671,8 +2965,32 @@
       <c r="E55" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F55" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I55" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J55" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K55" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L55" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M55" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A56" s="1" t="s">
         <v>65</v>
       </c>
@@ -1688,8 +3006,27 @@
       <c r="E56" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F56" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I56" s="5"/>
+      <c r="J56" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K56" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L56" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A57" s="1" t="s">
         <v>65</v>
       </c>
@@ -1705,8 +3042,32 @@
       <c r="E57" s="1">
         <v>80</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F57" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I57" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="J57" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K57" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L57" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M57" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A58" s="1" t="s">
         <v>65</v>
       </c>
@@ -1722,8 +3083,27 @@
       <c r="E58" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F58" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I58" s="5"/>
+      <c r="J58" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K58" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L58" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A59" s="1" t="s">
         <v>65</v>
       </c>
@@ -1739,8 +3119,27 @@
       <c r="E59" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F59" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G59" t="s">
+        <v>91</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I59" s="5"/>
+      <c r="J59" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K59" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L59" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A60" s="1" t="s">
         <v>65</v>
       </c>
@@ -1756,8 +3155,32 @@
       <c r="E60" s="1">
         <v>40</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F60" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I60" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="J60" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K60" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L60" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M60" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A61" s="1" t="s">
         <v>65</v>
       </c>
@@ -1773,8 +3196,32 @@
       <c r="E61" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F61" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H61" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I61" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="J61" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K61" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L61" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="M61" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A62" s="1" t="s">
         <v>65</v>
       </c>
@@ -1790,8 +3237,32 @@
       <c r="E62" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F62" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H62" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I62" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="J62" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K62" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L62" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M62" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A63" s="1" t="s">
         <v>65</v>
       </c>
@@ -1807,8 +3278,32 @@
       <c r="E63" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F63" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I63" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="J63" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K63" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L63" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M63" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A64" s="1" t="s">
         <v>65</v>
       </c>
@@ -1824,8 +3319,29 @@
       <c r="E64" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F64" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H64" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I64" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="J64" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K64" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L64" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A65" s="1" t="s">
         <v>65</v>
       </c>
@@ -1841,8 +3357,27 @@
       <c r="E65" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F65" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H65" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I65" s="4"/>
+      <c r="J65" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K65" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L65" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A66" s="2" t="s">
         <v>22</v>
       </c>
@@ -1858,8 +3393,27 @@
       <c r="E66" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F66" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H66" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I66" s="5"/>
+      <c r="J66" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L66" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A67" s="2" t="s">
         <v>22</v>
       </c>
@@ -1875,8 +3429,27 @@
       <c r="E67" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F67" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H67" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I67" s="5"/>
+      <c r="J67" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K67" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L67" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A68" s="1" t="s">
         <v>76</v>
       </c>
@@ -1892,8 +3465,27 @@
       <c r="E68" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F68" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H68" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I68" s="4"/>
+      <c r="J68" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K68" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L68" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A69" s="1" t="s">
         <v>76</v>
       </c>
@@ -1909,8 +3501,32 @@
       <c r="E69" s="1">
         <v>80</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F69" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H69" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I69" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="J69" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K69" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L69" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M69" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A70" s="1" t="s">
         <v>76</v>
       </c>
@@ -1926,8 +3542,27 @@
       <c r="E70" s="1">
         <v>48</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F70" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H70" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I70" s="4"/>
+      <c r="J70" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K70" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L70" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A71" s="2" t="s">
         <v>78</v>
       </c>
@@ -1943,8 +3578,27 @@
       <c r="E71" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F71" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H71" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I71" s="4"/>
+      <c r="J71" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K71" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L71" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A72" s="2" t="s">
         <v>78</v>
       </c>
@@ -1960,8 +3614,32 @@
       <c r="E72" s="2">
         <v>80</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F72" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I72" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="J72" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K72" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L72" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M72" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A73" s="2" t="s">
         <v>78</v>
       </c>
@@ -1977,8 +3655,32 @@
       <c r="E73" s="2">
         <v>60</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F73" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I73" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="J73" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K73" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L73" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M73" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A74" s="2" t="s">
         <v>78</v>
       </c>
@@ -1994,8 +3696,29 @@
       <c r="E74" s="2">
         <v>60</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F74" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I74" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="J74" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K74" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L74" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A75" s="2" t="s">
         <v>78</v>
       </c>
@@ -2011,8 +3734,27 @@
       <c r="E75" s="2">
         <v>120</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F75" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I75" s="4"/>
+      <c r="J75" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K75" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L75" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A76" s="2" t="s">
         <v>78</v>
       </c>
@@ -2028,8 +3770,32 @@
       <c r="E76" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F76" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I76" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K76" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L76" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M76" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A77" s="2" t="s">
         <v>78</v>
       </c>
@@ -2045,8 +3811,32 @@
       <c r="E77" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F77" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I77" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="J77" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K77" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L77" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M77" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A78" s="2" t="s">
         <v>78</v>
       </c>
@@ -2062,8 +3852,29 @@
       <c r="E78" s="2">
         <v>20</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F78" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H78" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I78" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="J78" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K78" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L78" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A79" s="2" t="s">
         <v>78</v>
       </c>
@@ -2079,8 +3890,32 @@
       <c r="E79" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F79" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H79" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I79" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="J79" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K79" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L79" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M79" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A80" s="2" t="s">
         <v>78</v>
       </c>
@@ -2096,8 +3931,27 @@
       <c r="E80" s="2">
         <v>48</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F80" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I80" s="4"/>
+      <c r="J80" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K80" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L80" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A81" s="2" t="s">
         <v>78</v>
       </c>
@@ -2113,8 +3967,27 @@
       <c r="E81" s="2">
         <v>48</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F81" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I81" s="4"/>
+      <c r="J81" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K81" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L81" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A82" s="2" t="s">
         <v>78</v>
       </c>
@@ -2130,8 +4003,27 @@
       <c r="E82" s="2">
         <v>16</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F82" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H82" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I82" s="4"/>
+      <c r="J82" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K82" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L82" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A83" s="1" t="s">
         <v>80</v>
       </c>
@@ -2147,8 +4039,27 @@
       <c r="E83" s="1">
         <v>40</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F83" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I83" s="4"/>
+      <c r="J83" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K83" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L83" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A84" s="1" t="s">
         <v>80</v>
       </c>
@@ -2164,8 +4075,27 @@
       <c r="E84" s="1">
         <v>100</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F84" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I84" s="4"/>
+      <c r="J84" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K84" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L84" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A85" s="1" t="s">
         <v>80</v>
       </c>
@@ -2180,6 +4110,25 @@
       </c>
       <c r="E85" s="1">
         <v>4</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H85" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I85" s="4"/>
+      <c r="J85" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K85" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L85" s="1" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -2188,25 +4137,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <MediaLengthInSeconds xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CA5D0A6329BB324E86983B32928CFC2E" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d7eac4bce3bbb09c82bd908806be82e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xmlns:ns3="ced60a7f-99b1-48d2-b555-34851c8026ae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb51570e5b7cb8bd524bc2df5324d4a3" ns2:_="" ns3:_="">
     <xsd:import namespace="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
@@ -2447,6 +4377,25 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <MediaLengthInSeconds xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2457,17 +4406,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB560F9-4CC1-4243-8F16-7FDC2CD703FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ced60a7f-99b1-48d2-b555-34851c8026ae"/>
-    <ds:schemaRef ds:uri="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA285021-94D7-4152-B2E7-B2D9504C2DBD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2486,6 +4424,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB560F9-4CC1-4243-8F16-7FDC2CD703FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ced60a7f-99b1-48d2-b555-34851c8026ae"/>
+    <ds:schemaRef ds:uri="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0257D61C-6042-483B-9C34-3DE0D82CB154}">
   <ds:schemaRefs>

</xml_diff>